<commit_message>
feat: add comprehensive test scenarios for New Article
</commit_message>
<xml_diff>
--- a/Testdata/testdata_article.xlsx
+++ b/Testdata/testdata_article.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,12 +461,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>user_a</t>
+          <t>user_full</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>user_a@example.com</t>
+          <t>full@example.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -476,22 +476,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Article A</t>
+          <t>Full Article Title</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Desc A</t>
+          <t>Full Description</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Body A</t>
+          <t>Full Body Content</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>tag1</t>
+          <t>tag1, tag2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -503,37 +503,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>user_b</t>
+          <t>user_no_tags</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>user_b@example.com</t>
+          <t>notags@example.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pass456</t>
+          <t>pass123</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Article B</t>
+          <t>No Tags Title</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Desc B</t>
+          <t>No Tags Description</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Body B</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>tag2</t>
+          <t>No Tags Body</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -542,7 +537,183 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>user_no_desc</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>nodesc@example.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pass123</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>No Description Title</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>No Description Body</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>tag3</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>user_no_title</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>notitle@example.com</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>pass123</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Missing Title Desc</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Missing Title Body</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>tag4</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>user_no_body</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>nobody@example.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>pass123</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Missing Body Title</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Missing Body Desc</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>tag5</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>user_special</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>special@example.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>pass123</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Title: @#$%^&amp;*()!</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Desc: 🚀 emojis</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t># Markdown Header
+- list item</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>tag_!@#</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>user_all_empty</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>allempty@example.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pass123</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>